<commit_message>
update battery-swap decision model v4_3 (2026-09-02 audit refactor: capex/depreciation fix, claude new artifact)
</commit_message>
<xml_diff>
--- a/业务/换电/定量计算/换电战略决策模型_v4_3/outputs/换电决策树_v4.3.xlsx
+++ b/业务/换电/定量计算/换电战略决策模型_v4_3/outputs/换电决策树_v4.3.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="决策树" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="决策树" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3397,13 +3397,13 @@
         </is>
       </c>
       <c r="C95" s="2" t="n">
-        <v>1.2249</v>
+        <v>0.9185</v>
       </c>
       <c r="D95" s="2" t="n">
-        <v>1.4762</v>
+        <v>1.141</v>
       </c>
       <c r="E95" s="2" t="n">
-        <v>1.664</v>
+        <v>1.3182</v>
       </c>
       <c r="F95" s="2" t="inlineStr"/>
       <c r="G95" s="2" t="inlineStr">
@@ -3424,13 +3424,13 @@
         </is>
       </c>
       <c r="C96" s="2" t="n">
-        <v>1.2249</v>
+        <v>0.9185</v>
       </c>
       <c r="D96" s="2" t="n">
-        <v>1.4762</v>
+        <v>1.141</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>1.664</v>
+        <v>1.3182</v>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
@@ -3486,13 +3486,13 @@
         </is>
       </c>
       <c r="C98" s="2" t="n">
-        <v>521.7145</v>
+        <v>695.7252</v>
       </c>
       <c r="D98" s="2" t="n">
-        <v>576.0709000000001</v>
+        <v>745.3097</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>647.5395</v>
+        <v>817.3876</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
@@ -3517,13 +3517,13 @@
         </is>
       </c>
       <c r="C99" s="2" t="n">
-        <v>-216.2839</v>
+        <v>305.7481</v>
       </c>
       <c r="D99" s="2" t="n">
-        <v>0.2522</v>
+        <v>507.9686</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>207.6193</v>
+        <v>717.1636</v>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
@@ -3579,13 +3579,13 @@
         </is>
       </c>
       <c r="C101" s="2" t="n">
-        <v>855.3108999999999</v>
+        <v>333.2788</v>
       </c>
       <c r="D101" s="2" t="n">
-        <v>850.1623</v>
+        <v>342.446</v>
       </c>
       <c r="E101" s="2" t="n">
-        <v>869.8559</v>
+        <v>360.3116</v>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
@@ -3610,13 +3610,13 @@
         </is>
       </c>
       <c r="C102" s="2" t="n">
-        <v>833.0722</v>
+        <v>311.0402</v>
       </c>
       <c r="D102" s="2" t="n">
-        <v>827.9236</v>
+        <v>320.2073</v>
       </c>
       <c r="E102" s="2" t="n">
-        <v>847.6172</v>
+        <v>338.0729</v>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
@@ -3769,13 +3769,13 @@
         </is>
       </c>
       <c r="C107" s="2" t="n">
-        <v>7.2308</v>
+        <v>5.8692</v>
       </c>
       <c r="D107" s="2" t="n">
-        <v>6.6662</v>
+        <v>5.6711</v>
       </c>
       <c r="E107" s="2" t="n">
-        <v>6.3455</v>
+        <v>5.5573</v>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
@@ -3800,13 +3800,13 @@
         </is>
       </c>
       <c r="C108" s="2" t="n">
-        <v>4620.653</v>
+        <v>3750.5995</v>
       </c>
       <c r="D108" s="2" t="n">
-        <v>5669.0098</v>
+        <v>4822.8159</v>
       </c>
       <c r="E108" s="2" t="n">
-        <v>6837.1358</v>
+        <v>5987.8953</v>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
@@ -3831,13 +3831,13 @@
         </is>
       </c>
       <c r="C109" s="2" t="n">
-        <v>693.0979</v>
+        <v>562.5898999999999</v>
       </c>
       <c r="D109" s="2" t="n">
-        <v>850.3515</v>
+        <v>723.4224</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>1025.5704</v>
+        <v>898.1843</v>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
@@ -3924,13 +3924,13 @@
         </is>
       </c>
       <c r="C112" s="2" t="n">
-        <v>2.4894</v>
+        <v>3.0668</v>
       </c>
       <c r="D112" s="2" t="n">
-        <v>2.7002</v>
+        <v>3.174</v>
       </c>
       <c r="E112" s="2" t="n">
-        <v>2.8366</v>
+        <v>3.239</v>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
@@ -3990,13 +3990,13 @@
         </is>
       </c>
       <c r="C114" s="2" t="n">
-        <v>7.2308</v>
+        <v>5.8692</v>
       </c>
       <c r="D114" s="2" t="n">
-        <v>6.6662</v>
+        <v>5.6711</v>
       </c>
       <c r="E114" s="2" t="n">
-        <v>6.3455</v>
+        <v>5.5573</v>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>

</xml_diff>